<commit_message>
Republish Augsburg_2026_WC: Kayak Cross individual (Time Trials) RANK from official classification (124 cells; maintainer 2026-10-21)
</commit_message>
<xml_diff>
--- a/events/Augsburg_2026_WC/Augsburg_2026_WC_start.xlsx
+++ b/events/Augsburg_2026_WC/Augsburg_2026_WC_start.xlsx
@@ -18803,6 +18803,11 @@
       <c r="K308" t="n">
         <v>307</v>
       </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R308" t="inlineStr">
         <is>
           <t>COCHRANE Georgina</t>
@@ -18866,6 +18871,11 @@
       <c r="K309" t="n">
         <v>308</v>
       </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R309" t="inlineStr">
         <is>
           <t>ONOZAWA Mine</t>
@@ -18929,6 +18939,11 @@
       <c r="K310" t="n">
         <v>309</v>
       </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R310" t="inlineStr">
         <is>
           <t>XU Linxi</t>
@@ -18992,6 +19007,11 @@
       <c r="K311" t="n">
         <v>310</v>
       </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R311" t="inlineStr">
         <is>
           <t>ITO Kurumi</t>
@@ -19055,6 +19075,11 @@
       <c r="K312" t="n">
         <v>311</v>
       </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R312" t="inlineStr">
         <is>
           <t>MILLER Ellis</t>
@@ -19118,6 +19143,11 @@
       <c r="K313" t="n">
         <v>312</v>
       </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R313" t="inlineStr">
         <is>
           <t>PISTONI Lucia</t>
@@ -19181,6 +19211,11 @@
       <c r="K314" t="n">
         <v>313</v>
       </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R314" t="inlineStr">
         <is>
           <t>MINTALOVA Eliska</t>
@@ -19244,6 +19279,11 @@
       <c r="K315" t="n">
         <v>314</v>
       </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R315" t="inlineStr">
         <is>
           <t>SOKOLOVA Mariia</t>
@@ -19307,6 +19347,11 @@
       <c r="K316" t="n">
         <v>315</v>
       </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R316" t="inlineStr">
         <is>
           <t>CULLWICK Kahlia</t>
@@ -19370,6 +19415,11 @@
       <c r="K317" t="n">
         <v>316</v>
       </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="R317" t="inlineStr">
         <is>
           <t>KRYLOVA Kseniia</t>
@@ -19433,6 +19483,11 @@
       <c r="K318" t="n">
         <v>317</v>
       </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R318" t="inlineStr">
         <is>
           <t>BETTERIDGE Lois</t>
@@ -19496,6 +19551,11 @@
       <c r="K319" t="n">
         <v>318</v>
       </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R319" t="inlineStr">
         <is>
           <t>PITCHER FARRELL Cleo</t>
@@ -19559,6 +19619,11 @@
       <c r="K320" t="n">
         <v>319</v>
       </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="R320" t="inlineStr">
         <is>
           <t>OLSON Beatrice</t>
@@ -19685,6 +19750,11 @@
       <c r="K322" t="n">
         <v>321</v>
       </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R322" t="inlineStr">
         <is>
           <t>YAZAWA Aki</t>
@@ -19748,6 +19818,11 @@
       <c r="K323" t="n">
         <v>322</v>
       </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="R323" t="inlineStr">
         <is>
           <t>ANANYEVA Anastassiya</t>
@@ -19811,6 +19886,11 @@
       <c r="K324" t="n">
         <v>323</v>
       </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R324" t="inlineStr">
         <is>
           <t>BUETIKOFER Fia</t>
@@ -19874,6 +19954,11 @@
       <c r="K325" t="n">
         <v>324</v>
       </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R325" t="inlineStr">
         <is>
           <t>MACKIE Ada</t>
@@ -19937,6 +20022,11 @@
       <c r="K326" t="n">
         <v>325</v>
       </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R326" t="inlineStr">
         <is>
           <t>MICHALOVA Tereza</t>
@@ -20000,6 +20090,11 @@
       <c r="K327" t="n">
         <v>326</v>
       </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R327" t="inlineStr">
         <is>
           <t>MATTI Svenja</t>
@@ -20063,6 +20158,11 @@
       <c r="K328" t="n">
         <v>327</v>
       </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R328" t="inlineStr">
         <is>
           <t>DELASSUS Marjorie</t>
@@ -20126,6 +20226,11 @@
       <c r="K329" t="n">
         <v>328</v>
       </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R329" t="inlineStr">
         <is>
           <t>MINAZOVA Alsu</t>
@@ -20189,6 +20294,11 @@
       <c r="K330" t="n">
         <v>329</v>
       </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R330" t="inlineStr">
         <is>
           <t>BRZESKA Dominika</t>
@@ -20252,6 +20362,11 @@
       <c r="K331" t="n">
         <v>330</v>
       </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R331" t="inlineStr">
         <is>
           <t>ALTMAN Isabella</t>
@@ -20315,6 +20430,11 @@
       <c r="K332" t="n">
         <v>331</v>
       </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R332" t="inlineStr">
         <is>
           <t>PLOCHMANN Annkatrin</t>
@@ -20378,6 +20498,11 @@
       <c r="K333" t="n">
         <v>332</v>
       </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R333" t="inlineStr">
         <is>
           <t>GONI Leire</t>
@@ -20441,6 +20566,11 @@
       <c r="K334" t="n">
         <v>333</v>
       </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R334" t="inlineStr">
         <is>
           <t>CHEN Lin</t>
@@ -20504,6 +20634,11 @@
       <c r="K335" t="n">
         <v>334</v>
       </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="R335" t="inlineStr">
         <is>
           <t>PINTERIC Naja</t>
@@ -20567,6 +20702,11 @@
       <c r="K336" t="n">
         <v>335</v>
       </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R336" t="inlineStr">
         <is>
           <t>STANOVSKA Sona</t>
@@ -20630,6 +20770,11 @@
       <c r="K337" t="n">
         <v>336</v>
       </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="R337" t="inlineStr">
         <is>
           <t>REX Rosie</t>
@@ -20693,6 +20838,11 @@
       <c r="K338" t="n">
         <v>337</v>
       </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R338" t="inlineStr">
         <is>
           <t>ALTMAN Marcella</t>
@@ -20756,6 +20906,11 @@
       <c r="K339" t="n">
         <v>338</v>
       </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R339" t="inlineStr">
         <is>
           <t>HOCEVAR Eva Alina</t>
@@ -20882,6 +21037,11 @@
       <c r="K341" t="n">
         <v>340</v>
       </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R341" t="inlineStr">
         <is>
           <t>FOX Jessica</t>
@@ -20945,6 +21105,11 @@
       <c r="K342" t="n">
         <v>341</v>
       </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R342" t="inlineStr">
         <is>
           <t>LI Shiting</t>
@@ -21008,6 +21173,11 @@
       <c r="K343" t="n">
         <v>342</v>
       </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R343" t="inlineStr">
         <is>
           <t>TEUNISSEN Lena</t>
@@ -21071,6 +21241,11 @@
       <c r="K344" t="n">
         <v>343</v>
       </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R344" t="inlineStr">
         <is>
           <t>LAZKANO Miren</t>
@@ -21134,6 +21309,11 @@
       <c r="K345" t="n">
         <v>344</v>
       </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R345" t="inlineStr">
         <is>
           <t>LEAVER Lois</t>
@@ -21197,6 +21377,11 @@
       <c r="K346" t="n">
         <v>345</v>
       </c>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R346" t="inlineStr">
         <is>
           <t>SABATTINI Chiara</t>
@@ -21260,6 +21445,11 @@
       <c r="K347" t="n">
         <v>346</v>
       </c>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="R347" t="inlineStr">
         <is>
           <t>US Viktoriia</t>
@@ -21323,6 +21513,11 @@
       <c r="K348" t="n">
         <v>347</v>
       </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R348" t="inlineStr">
         <is>
           <t>ESTACIA NETA Omira</t>
@@ -21386,6 +21581,11 @@
       <c r="K349" t="n">
         <v>348</v>
       </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R349" t="inlineStr">
         <is>
           <t>BEKOVA Katerina</t>
@@ -21449,6 +21649,11 @@
       <c r="K350" t="n">
         <v>349</v>
       </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R350" t="inlineStr">
         <is>
           <t>HERZOG Andrea</t>
@@ -21512,6 +21717,11 @@
       <c r="K351" t="n">
         <v>350</v>
       </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R351" t="inlineStr">
         <is>
           <t>DORIA Monica</t>
@@ -21575,6 +21785,11 @@
       <c r="K352" t="n">
         <v>351</v>
       </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R352" t="inlineStr">
         <is>
           <t>SETCHELL Nikita</t>
@@ -21638,6 +21853,11 @@
       <c r="K353" t="n">
         <v>352</v>
       </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R353" t="inlineStr">
         <is>
           <t>SATILA Ana</t>
@@ -21701,6 +21921,11 @@
       <c r="K354" t="n">
         <v>353</v>
       </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R354" t="inlineStr">
         <is>
           <t>KNEBLOVA Tereza</t>
@@ -21764,6 +21989,11 @@
       <c r="K355" t="n">
         <v>354</v>
       </c>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R355" t="inlineStr">
         <is>
           <t>ZWOLINSKA Klaudia</t>
@@ -21827,6 +22057,11 @@
       <c r="K356" t="n">
         <v>355</v>
       </c>
+      <c r="M356" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R356" t="inlineStr">
         <is>
           <t>FOX Noemie</t>
@@ -21890,6 +22125,11 @@
       <c r="K357" t="n">
         <v>356</v>
       </c>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R357" t="inlineStr">
         <is>
           <t>MARX Alena</t>
@@ -21953,6 +22193,11 @@
       <c r="K358" t="n">
         <v>357</v>
       </c>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R358" t="inlineStr">
         <is>
           <t>FUNK Ricarda</t>
@@ -22016,6 +22261,11 @@
       <c r="K359" t="n">
         <v>358</v>
       </c>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R359" t="inlineStr">
         <is>
           <t>CHOURRAUT Maialen</t>
@@ -22079,6 +22329,11 @@
       <c r="K360" t="n">
         <v>359</v>
       </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R360" t="inlineStr">
         <is>
           <t>LEIBFARTH Evy</t>
@@ -22142,6 +22397,11 @@
       <c r="K361" t="n">
         <v>360</v>
       </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R361" t="inlineStr">
         <is>
           <t>PRIGENT Camille</t>
@@ -22205,6 +22465,11 @@
       <c r="K362" t="n">
         <v>361</v>
       </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R362" t="inlineStr">
         <is>
           <t>HUG Angele</t>
@@ -22268,6 +22533,11 @@
       <c r="K363" t="n">
         <v>362</v>
       </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R363" t="inlineStr">
         <is>
           <t>BROWN Ben</t>
@@ -22331,6 +22601,11 @@
       <c r="K364" t="n">
         <v>363</v>
       </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
       <c r="R364" t="inlineStr">
         <is>
           <t>ADACHI Kazuya</t>
@@ -22394,6 +22669,11 @@
       <c r="K365" t="n">
         <v>364</v>
       </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
       <c r="R365" t="inlineStr">
         <is>
           <t>OBLINGER Milo</t>
@@ -22457,6 +22737,11 @@
       <c r="K366" t="n">
         <v>365</v>
       </c>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
       <c r="R366" t="inlineStr">
         <is>
           <t>YALKIN Eren Hasan</t>
@@ -22520,6 +22805,11 @@
       <c r="K367" t="n">
         <v>366</v>
       </c>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="R367" t="inlineStr">
         <is>
           <t>PARRY Daniel</t>
@@ -22583,6 +22873,11 @@
       <c r="K368" t="n">
         <v>367</v>
       </c>
+      <c r="M368" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="R368" t="inlineStr">
         <is>
           <t>COWAN Padraig</t>
@@ -22646,6 +22941,11 @@
       <c r="K369" t="n">
         <v>368</v>
       </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R369" t="inlineStr">
         <is>
           <t>WENG Jize</t>
@@ -22709,6 +23009,11 @@
       <c r="K370" t="n">
         <v>369</v>
       </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="R370" t="inlineStr">
         <is>
           <t>ETTWILLER Gael</t>
@@ -22772,6 +23077,11 @@
       <c r="K371" t="n">
         <v>370</v>
       </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R371" t="inlineStr">
         <is>
           <t>HENDRICK Noel</t>
@@ -22835,6 +23145,11 @@
       <c r="K372" t="n">
         <v>371</v>
       </c>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
       <c r="R372" t="inlineStr">
         <is>
           <t>WESTFALL Tyler</t>
@@ -22898,6 +23213,11 @@
       <c r="K373" t="n">
         <v>372</v>
       </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
       <c r="R373" t="inlineStr">
         <is>
           <t>KONRAD Marten</t>
@@ -22961,6 +23281,11 @@
       <c r="K374" t="n">
         <v>373</v>
       </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R374" t="inlineStr">
         <is>
           <t>HELLO Joris</t>
@@ -23024,6 +23349,11 @@
       <c r="K375" t="n">
         <v>374</v>
       </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
       <c r="R375" t="inlineStr">
         <is>
           <t>SAYDULLAEV Samandar</t>
@@ -23150,6 +23480,11 @@
       <c r="K377" t="n">
         <v>376</v>
       </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R377" t="inlineStr">
         <is>
           <t>EGYHAZY Matus</t>
@@ -23213,6 +23548,11 @@
       <c r="K378" t="n">
         <v>377</v>
       </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R378" t="inlineStr">
         <is>
           <t>SMOLEN Michal</t>
@@ -23276,6 +23616,11 @@
       <c r="K379" t="n">
         <v>378</v>
       </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="R379" t="inlineStr">
         <is>
           <t>MARIEN Martin</t>
@@ -23339,6 +23684,11 @@
       <c r="K380" t="n">
         <v>379</v>
       </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="R380" t="inlineStr">
         <is>
           <t>ROZENTALS Klass Francisks</t>
@@ -23402,6 +23752,11 @@
       <c r="K381" t="n">
         <v>380</v>
       </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
       <c r="R381" t="inlineStr">
         <is>
           <t>BARAT Andy</t>
@@ -23465,6 +23820,11 @@
       <c r="K382" t="n">
         <v>381</v>
       </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
       <c r="R382" t="inlineStr">
         <is>
           <t>EGYHAZY Dominik</t>
@@ -23528,6 +23888,11 @@
       <c r="K383" t="n">
         <v>382</v>
       </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
       <c r="R383" t="inlineStr">
         <is>
           <t>MAGAN Raage</t>
@@ -23591,6 +23956,11 @@
       <c r="K384" t="n">
         <v>383</v>
       </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R384" t="inlineStr">
         <is>
           <t>TEMIRGALIEV Djanibek</t>
@@ -23654,6 +24024,11 @@
       <c r="K385" t="n">
         <v>384</v>
       </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R385" t="inlineStr">
         <is>
           <t>TANAKA Yuuki</t>
@@ -23717,6 +24092,11 @@
       <c r="K386" t="n">
         <v>385</v>
       </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R386" t="inlineStr">
         <is>
           <t>MUTO Yusuke</t>
@@ -23780,6 +24160,11 @@
       <c r="K387" t="n">
         <v>386</v>
       </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="R387" t="inlineStr">
         <is>
           <t>ANDERSON Finn</t>
@@ -23843,6 +24228,11 @@
       <c r="K388" t="n">
         <v>387</v>
       </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
       <c r="R388" t="inlineStr">
         <is>
           <t>UKALOVIC Thomas</t>
@@ -23906,6 +24296,11 @@
       <c r="K389" t="n">
         <v>388</v>
       </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="R389" t="inlineStr">
         <is>
           <t>DA SILVA Kaua</t>
@@ -23969,6 +24364,11 @@
       <c r="K390" t="n">
         <v>389</v>
       </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="R390" t="inlineStr">
         <is>
           <t>SOVKO Serhii</t>
@@ -24032,6 +24432,11 @@
       <c r="K391" t="n">
         <v>390</v>
       </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
       <c r="R391" t="inlineStr">
         <is>
           <t>KOROBOV Alexandr</t>
@@ -24095,6 +24500,11 @@
       <c r="K392" t="n">
         <v>391</v>
       </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R392" t="inlineStr">
         <is>
           <t>KRACHKO Arkhyp</t>
@@ -24158,6 +24568,11 @@
       <c r="K393" t="n">
         <v>392</v>
       </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R393" t="inlineStr">
         <is>
           <t>HAYLETT Ben</t>
@@ -24221,6 +24636,11 @@
       <c r="K394" t="n">
         <v>393</v>
       </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R394" t="inlineStr">
         <is>
           <t>EIGEL Pavel</t>
@@ -24284,6 +24704,11 @@
       <c r="K395" t="n">
         <v>394</v>
       </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R395" t="inlineStr">
         <is>
           <t>BRZEZINSKI Jakub</t>
@@ -24347,6 +24772,11 @@
       <c r="K396" t="n">
         <v>395</v>
       </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R396" t="inlineStr">
         <is>
           <t>SMIRNOV Egor</t>
@@ -24410,6 +24840,11 @@
       <c r="K397" t="n">
         <v>396</v>
       </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R397" t="inlineStr">
         <is>
           <t>FEDORENKO Oleksandr</t>
@@ -24473,6 +24908,11 @@
       <c r="K398" t="n">
         <v>397</v>
       </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R398" t="inlineStr">
         <is>
           <t>PISTONI Michele</t>
@@ -24536,6 +24976,11 @@
       <c r="K399" t="n">
         <v>398</v>
       </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R399" t="inlineStr">
         <is>
           <t>SACHERS Felix</t>
@@ -24599,6 +25044,11 @@
       <c r="K400" t="n">
         <v>399</v>
       </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R400" t="inlineStr">
         <is>
           <t>KOZLOV Ivan</t>
@@ -24662,6 +25112,11 @@
       <c r="K401" t="n">
         <v>400</v>
       </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R401" t="inlineStr">
         <is>
           <t>LEITNER Mario</t>
@@ -24725,6 +25180,11 @@
       <c r="K402" t="n">
         <v>401</v>
       </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="R402" t="inlineStr">
         <is>
           <t>GUTKNECHT Patrick</t>
@@ -24788,6 +25248,11 @@
       <c r="K403" t="n">
         <v>402</v>
       </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R403" t="inlineStr">
         <is>
           <t>CROSBEE Mark</t>
@@ -24851,6 +25316,11 @@
       <c r="K404" t="n">
         <v>403</v>
       </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R404" t="inlineStr">
         <is>
           <t>SAVLI Jakob</t>
@@ -24914,6 +25384,11 @@
       <c r="K405" t="n">
         <v>404</v>
       </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
       <c r="R405" t="inlineStr">
         <is>
           <t>ECHANIZ Pau</t>
@@ -24977,6 +25452,11 @@
       <c r="K406" t="n">
         <v>405</v>
       </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R406" t="inlineStr">
         <is>
           <t>ZIMMERMAN Isaac</t>
@@ -25040,6 +25520,11 @@
       <c r="K407" t="n">
         <v>406</v>
       </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R407" t="inlineStr">
         <is>
           <t>FERRAZZI Xabier</t>
@@ -25103,6 +25588,11 @@
       <c r="K408" t="n">
         <v>407</v>
       </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R408" t="inlineStr">
         <is>
           <t>OSCHMAUTZ Felix</t>
@@ -25166,6 +25656,11 @@
       <c r="K409" t="n">
         <v>408</v>
       </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R409" t="inlineStr">
         <is>
           <t>KUCHNO Tadeusz</t>
@@ -25229,6 +25724,11 @@
       <c r="K410" t="n">
         <v>409</v>
       </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R410" t="inlineStr">
         <is>
           <t>HENGST Stefan</t>
@@ -25292,6 +25792,11 @@
       <c r="K411" t="n">
         <v>410</v>
       </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R411" t="inlineStr">
         <is>
           <t>QUAN Xin</t>
@@ -25355,6 +25860,11 @@
       <c r="K412" t="n">
         <v>411</v>
       </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R412" t="inlineStr">
         <is>
           <t>HU Zhaoshan</t>
@@ -25418,6 +25928,11 @@
       <c r="K413" t="n">
         <v>412</v>
       </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R413" t="inlineStr">
         <is>
           <t>DE COSTER Gabriel</t>
@@ -25481,6 +25996,11 @@
       <c r="K414" t="n">
         <v>413</v>
       </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
       <c r="R414" t="inlineStr">
         <is>
           <t>BALDONI Alex</t>
@@ -25544,6 +26064,11 @@
       <c r="K415" t="n">
         <v>414</v>
       </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R415" t="inlineStr">
         <is>
           <t>RUDORFER Martin</t>
@@ -25607,6 +26132,11 @@
       <c r="K416" t="n">
         <v>415</v>
       </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R416" t="inlineStr">
         <is>
           <t>MARX Dimitri</t>
@@ -25670,6 +26200,11 @@
       <c r="K417" t="n">
         <v>416</v>
       </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R417" t="inlineStr">
         <is>
           <t>COLLIER Nicholas</t>
@@ -25733,6 +26268,11 @@
       <c r="K418" t="n">
         <v>417</v>
       </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R418" t="inlineStr">
         <is>
           <t>DELFOUR Lucien</t>
@@ -25796,6 +26336,11 @@
       <c r="K419" t="n">
         <v>418</v>
       </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R419" t="inlineStr">
         <is>
           <t>DE GENNARO Giovanni</t>
@@ -25859,6 +26404,11 @@
       <c r="K420" t="n">
         <v>419</v>
       </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R420" t="inlineStr">
         <is>
           <t>LLORENTE David</t>
@@ -25922,6 +26472,11 @@
       <c r="K421" t="n">
         <v>420</v>
       </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R421" t="inlineStr">
         <is>
           <t>RENIA Benjamin</t>
@@ -25985,6 +26540,11 @@
       <c r="K422" t="n">
         <v>421</v>
       </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R422" t="inlineStr">
         <is>
           <t>ROHRER Jan</t>
@@ -26048,6 +26608,11 @@
       <c r="K423" t="n">
         <v>422</v>
       </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R423" t="inlineStr">
         <is>
           <t>HOCEVAR Ziga Lin</t>
@@ -26111,6 +26676,11 @@
       <c r="K424" t="n">
         <v>423</v>
       </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="R424" t="inlineStr">
         <is>
           <t>LONG Merle</t>
@@ -26174,6 +26744,11 @@
       <c r="K425" t="n">
         <v>424</v>
       </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R425" t="inlineStr">
         <is>
           <t>AUBERTIN Maxime</t>
@@ -26237,6 +26812,11 @@
       <c r="K426" t="n">
         <v>425</v>
       </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R426" t="inlineStr">
         <is>
           <t>KREJCI Jakub</t>
@@ -26300,6 +26880,11 @@
       <c r="K427" t="n">
         <v>426</v>
       </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R427" t="inlineStr">
         <is>
           <t>LEAVER Sam</t>
@@ -26363,6 +26948,11 @@
       <c r="K428" t="n">
         <v>427</v>
       </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R428" t="inlineStr">
         <is>
           <t>GONCALVES Pedro</t>
@@ -26426,6 +27016,11 @@
       <c r="K429" t="n">
         <v>428</v>
       </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R429" t="inlineStr">
         <is>
           <t>OCHOA Manuel</t>
@@ -26489,6 +27084,11 @@
       <c r="K430" t="n">
         <v>429</v>
       </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R430" t="inlineStr">
         <is>
           <t>POLACZYK Mateusz</t>
@@ -26552,6 +27152,11 @@
       <c r="K431" t="n">
         <v>430</v>
       </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="R431" t="inlineStr">
         <is>
           <t>NOVAK Matyas</t>
@@ -26615,6 +27220,11 @@
       <c r="K432" t="n">
         <v>431</v>
       </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R432" t="inlineStr">
         <is>
           <t>MADORE Mathurin</t>
@@ -26678,6 +27288,11 @@
       <c r="K433" t="n">
         <v>432</v>
       </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R433" t="inlineStr">
         <is>
           <t>BUTCHER Finn</t>
@@ -26740,6 +27355,11 @@
       </c>
       <c r="K434" t="n">
         <v>433</v>
+      </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="R434" t="inlineStr">
         <is>

</xml_diff>